<commit_message>
update v3.1 and v3.2
</commit_message>
<xml_diff>
--- a/docs/revised_shatin/qwen3-next-80b-a3b-thinking/test_grammar_1_['No. 51_～と〈条件(じょうけん)〉 ']_revised_iteration_1.xlsx
+++ b/docs/revised_shatin/qwen3-next-80b-a3b-thinking/test_grammar_1_['No. 51_～と〈条件(じょうけん)〉 ']_revised_iteration_1.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F80"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -467,12 +467,12 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 朝ごはんを食べる (   )、元気になります。</t>
+          <t>: もんだい1雨が降る (   )、出かけません。</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>1. ので 2. から 3. と 4. たら</t>
+          <t>1. ので 2. と 3. から 4. たら</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -491,17 +491,17 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 この道をまっすぐ行く (   )、駅があります。</t>
+          <t>: もんだい1朝ごはんを食べる (   )、元気になります。</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>1. ので 2. と 3. から 4. たら</t>
+          <t>1. ので 2. から 3. と 4. たら</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr"/>
@@ -515,7 +515,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 右に曲がる (   )、スーパーがあります。</t>
+          <t>: もんだい1この道をまっすぐ行く (   )、駅があります。</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr"/>
@@ -539,7 +539,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 このボタンを押す (   )、ドアが開きます。</t>
+          <t>: もんだい1右に曲がる (   )、スーパーがあります。</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr"/>
@@ -563,7 +563,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 春になる (   )、花が咲きます。</t>
+          <t>: もんだい1このボタンを押す (   )、ドアが開きます。</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
@@ -573,7 +573,7 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr"/>
@@ -587,7 +587,7 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 勉強を頑張る (   )、試験に合格できます。</t>
+          <t>: もんだい1春になる (   )、花が咲きます。</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr"/>
@@ -611,7 +611,7 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 店に入る (   )、すぐに店員が来ました。</t>
+          <t>: もんだい1勉強を頑張る (   )、試験に合格できます。</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr"/>
@@ -635,15 +635,12 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 道を歩いている(   )、友達に会いました。</t>
+          <t>: もんだい1店に入る (   )、すぐに店員が来ました。</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>1. たら
-2. と
-3. て
-4. で</t>
+          <t>1. ので 2. と 3. から 4. たら</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
@@ -662,7 +659,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 ボタンを押す (   )、電気が消えます。</t>
+          <t>: もんだい1道を歩いている (   )、友達に会いました。</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
@@ -672,7 +669,7 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr"/>
@@ -686,12 +683,12 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 私は 朝 起きる (   )、まず コーヒーを 飲みます。</t>
+          <t>: もんだい1ボタンを押す (   )、電気が消えます。</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>1. に 2. と 3. で 4. が</t>
+          <t>1. ので 2. と 3. から 4. たら</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
@@ -710,17 +707,17 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 このボタンを 押す (   )、ドアが 開きます。</t>
+          <t>: もんだい2私は 朝 起きる (   )、まず コーヒーを 飲みます。</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>1. を 2. で 3. と 4. に</t>
+          <t>1. に 2. と 3. で 4. が</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr"/>
@@ -734,17 +731,17 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 雨が 降る (   )、試合は 中止になります。</t>
+          <t>: もんだい2このボタンを 押す (   )、ドアが 開きます。</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>1. が 2. と 3. に 4. を</t>
+          <t>1. を 2. で 3. と 4. に</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr"/>
@@ -758,17 +755,17 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 彼は 家に 帰る (   )、すぐに 寝ます。</t>
+          <t>: もんだい2雨が 降る (   )、試合は 中止になります。</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>1. と 2. で 3. に 4. が</t>
+          <t>1. が 2. と 3. に 4. を</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr"/>
@@ -782,17 +779,17 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 ボタンを 押す (   )、音楽が 流れます。</t>
+          <t>: もんだい2彼は 家に 帰る (   )、すぐに 寝ます。</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>1. で 2. に 3. と 4. が</t>
+          <t>1. と 2. で 3. に 4. が</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr"/>
@@ -806,17 +803,17 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 この道を まっすぐ 行く (   )、駅に 着きます。</t>
+          <t>: もんだい2ボタンを 押す (   )、音楽が 流れます。</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>1. が 2. と 3. に 4. で</t>
+          <t>1. で 2. に 3. と 4. が</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr"/>
@@ -830,12 +827,12 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 春が 来る (   )、桜が 咲きます。</t>
+          <t>: もんだい2この道を まっすぐ 行く (   )、駅に 着きます。</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>1. に 2. と 3. が 4. で</t>
+          <t>1. が 2. と 3. に 4. で</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
@@ -854,17 +851,17 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 信号が 青に なる (   )、渡りましょう。</t>
+          <t>: もんだい2春が 来る (   )、桜が 咲きます。</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>1. で 2. に 3. と 4. が</t>
+          <t>1. に 2. と 3. が 4. で</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr"/>
@@ -878,17 +875,17 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 電車が 来る (   )、ホームに 並びます。</t>
+          <t>: もんだい2信号が 青に なる (   )、渡りましょう。</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>1. を 2. と 3. が 4. に</t>
+          <t>1. で 2. に 3. と 4. が</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E19" s="1" t="inlineStr"/>
@@ -902,17 +899,17 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 この薬を 飲む (   )、頭痛が 治ります。</t>
+          <t>: もんだい2電車が 来る (   )、ホームに 並びます。</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>1. と 2. に 3. で 4. が</t>
+          <t>1. を 2. と 3. が 4. に</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr"/>
@@ -926,12 +923,12 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 天気予報によると、明日は雨が(   )そうです。</t>
+          <t>: もんだい2この薬を 飲む (   )、頭痛が 治ります。</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>1. ふる 2. ふって 3. ふらない 4. ふった</t>
+          <t>1. と 2. に 3. で 4. が</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr">
@@ -950,12 +947,12 @@
       </c>
       <c r="B22" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 このボタンを押すと、テレビが(   )。</t>
+          <t>: もんだい3天気予報によると、明日は雨が(   )そうです。</t>
         </is>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>1. つく 2. つける 3. ついて 4. つかない</t>
+          <t>1. ふる 2. ふって 3. ふらない 4. ふった</t>
         </is>
       </c>
       <c r="D22" s="1" t="inlineStr">
@@ -974,17 +971,17 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 先生の話を聞くと、(   )ことが多いです。</t>
+          <t>: もんだい3このボタンを押すと、テレビが(   )。</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>1. 学ぶ 2. 学び 3. 学んだ 4. 学んで</t>
+          <t>1. つく 2. つける 3. ついて 4. つかない</t>
         </is>
       </c>
       <c r="D23" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E23" s="1" t="inlineStr"/>
@@ -998,17 +995,17 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 この道をまっすぐ行くと、駅が(   )。</t>
+          <t>: もんだい3先生の話を聞くと、(   )ことが多いです。</t>
         </is>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>1. ある 2. あり 3. あって 4. ない</t>
+          <t>1. 学ぶ 2. 学び 3. 学んだ 4. 学んで</t>
         </is>
       </c>
       <c r="D24" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E24" s="1" t="inlineStr"/>
@@ -1022,12 +1019,12 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 お金がないと、(   )ことができません。</t>
+          <t>: もんだい3この道をまっすぐ行くと、駅が(   )。</t>
         </is>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
-          <t>1. 買う 2. 買い 3. 買って 4. 買わない</t>
+          <t>1. ある 2. あり 3. あって 4. ない</t>
         </is>
       </c>
       <c r="D25" s="1" t="inlineStr">
@@ -1046,17 +1043,17 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 夏になると、(   )が食べたくなります。</t>
+          <t>: もんだい3お金がないと、(   )ことができません。</t>
         </is>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>1. すいか 2. すいかを 3. すいかの 4. すいかが</t>
+          <t>1. 買う 2. 買い 3. 買って 4. 買わない</t>
         </is>
       </c>
       <c r="D26" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E26" s="1" t="inlineStr"/>
@@ -1070,17 +1067,17 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 この本を読むと、(   )が広がります。</t>
+          <t>: もんだい3夏になると、(   )が食べたくなります。</t>
         </is>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>1. しりょう 2. しりょうの 3. しりょうが 4. しりょうを</t>
+          <t>1. すいか 2. すいかを 3. すいかの 4. すいかが</t>
         </is>
       </c>
       <c r="D27" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E27" s="1" t="inlineStr"/>
@@ -1094,17 +1091,17 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 友達に会うと、いつも(   )。</t>
+          <t>: もんだい3この本を読むと、(   )が広がります。</t>
         </is>
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>1. 楽しい 2. 楽しんで 3. 楽しむ 4. 楽しそう</t>
+          <t>1. しりょう 2. しりょうの 3. しりょうが 4. しりょうを</t>
         </is>
       </c>
       <c r="D28" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E28" s="1" t="inlineStr"/>
@@ -1118,17 +1115,17 @@
       </c>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 家を出ると、すぐに雨が(   )。</t>
+          <t>: もんだい3友達に会うと、いつも(   )。</t>
         </is>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>1. ふる 2. ふって 3. ふり 4. ふった</t>
+          <t>1. 楽しい 2. 楽しんで 3. 楽しむ 4. 楽しそう</t>
         </is>
       </c>
       <c r="D29" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E29" s="1" t="inlineStr"/>
@@ -1142,12 +1139,12 @@
       </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>: もんだい3 この薬を飲むと、頭痛が(   )。</t>
+          <t>: もんだい3家を出ると、すぐに雨が(   )。</t>
         </is>
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>1. なおる 2. なおり 3. なおって 4. なおらない</t>
+          <t>1. ふる 2. ふって 3. ふり 4. ふった</t>
         </is>
       </c>
       <c r="D30" s="1" t="inlineStr">
@@ -1166,17 +1163,17 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 もし 雨が 降ったら、 ピクニックは (   ).</t>
+          <t>: もんだい3この薬を飲むと、頭痛が(   )。</t>
         </is>
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
-          <t>1. 行くことにした 2. 行けないかもしれない 3. 行きたくない 4. 行くつもりだ</t>
+          <t>1. なおる 2. なおり 3. なおって 4. なおらない</t>
         </is>
       </c>
       <c r="D31" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E31" s="1" t="inlineStr"/>
@@ -1190,17 +1187,17 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 財布を 忘れると、 買い物が (   ).</t>
+          <t>: もんだい4もし 雨が 降ったら、 ピクニックは (   ).</t>
         </is>
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t>1. できないかもしれない 2. できることにした 3. できないそうだ 4. できたかった</t>
+          <t>1. 行くことにした 2. 行けないかもしれない 3. 行きたくない 4. 行くつもりだ</t>
         </is>
       </c>
       <c r="D32" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E32" s="1" t="inlineStr"/>
@@ -1214,12 +1211,12 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 もし 試験に 合格したら、 新しいパソコンを (   ).</t>
+          <t>: もんだい4財布を 忘れると、 買い物が (   ).</t>
         </is>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>1. 買いたい 2. 買うことにした 3. 買いたがっている 4. 買いそうだ</t>
+          <t>1. できないかもしれない 2. できることにした 3. できないそうだ 4. できたかった</t>
         </is>
       </c>
       <c r="D33" s="1" t="inlineStr">
@@ -1238,17 +1235,17 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 彼女に 会うと、 いつも (   ).</t>
+          <t>: もんだい4もし 試験に 合格したら、 新しいパソコンを (   ).</t>
         </is>
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>1. うれしいだろう 2. うれしいことにした 3. うれしいそうだ 4. うれしくなる</t>
+          <t>1. 買いたい 2. 買うことにした 3. 買いたがっている 4. 買いそうだ</t>
         </is>
       </c>
       <c r="D34" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E34" s="1" t="inlineStr"/>
@@ -1262,17 +1259,17 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 もし 時間が あったら、 一緒に 映画を (   ).</t>
+          <t>: もんだい4彼女に 会うと、 いつも (   ).</t>
         </is>
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t>1. 見ることにした 2. 見ようと思う 3. 見たいかもしれない 4. 見るらしい</t>
+          <t>1. うれしいだろう 2. うれしいことにした 3. うれしいそうだ 4. うれしくなる</t>
         </is>
       </c>
       <c r="D35" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E35" s="1" t="inlineStr"/>
@@ -1286,17 +1283,17 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 宿題を 終わらせると、 友達と (   ).</t>
+          <t>: もんだい4もし 時間が あったら、 一緒に 映画を (   ).</t>
         </is>
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t>1. 遊びたい 2. 遊びに行くことにした 3. 遊ぶかもしれない 4. 遊びたがる</t>
+          <t>1. 見ることにした 2. 見ようと思う 3. 見たいかもしれない 4. 見るらしい</t>
         </is>
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E36" s="1" t="inlineStr"/>
@@ -1310,12 +1307,12 @@
       </c>
       <c r="B37" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 もし 電車が 遅れたら、 タクシーで (   ).</t>
+          <t>: もんだい4宿題を 終わらせると、 友達と (   ).</t>
         </is>
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t>1. 行くつもりだ 2. 行くことにした 3. 行きたいと思う 4. 行くようになった</t>
+          <t>1. 遊びたい 2. 遊びに行くことにした 3. 遊ぶかもしれない 4. 遊びたがる</t>
         </is>
       </c>
       <c r="D37" s="1" t="inlineStr">
@@ -1334,17 +1331,17 @@
       </c>
       <c r="B38" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 彼に 会ったら、 すぐに (   ).</t>
+          <t>: もんだい4もし 電車が 遅れたら、 タクシーで (   ).</t>
         </is>
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
-          <t>1. 話すことにした 2. 話したいと思う 3. 話せるらしい 4. 話しそうだ</t>
+          <t>1. 行くつもりだ 2. 行くことにした 3. 行きたいと思う 4. 行くようになった</t>
         </is>
       </c>
       <c r="D38" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E38" s="1" t="inlineStr"/>
@@ -1358,17 +1355,17 @@
       </c>
       <c r="B39" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 もし お金が 足りなかったら、 アルバイトを (   ).</t>
+          <t>: もんだい4彼に 会ったら、 すぐに (   ).</t>
         </is>
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t>1. することにした 2. したいかもしれない 3. するようになった 4. したらしい</t>
+          <t>1. 話すことにした 2. 話したいと思う 3. 話せるらしい 4. 話しそうだ</t>
         </is>
       </c>
       <c r="D39" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E39" s="1" t="inlineStr"/>
@@ -1382,17 +1379,17 @@
       </c>
       <c r="B40" s="1" t="inlineStr">
         <is>
-          <t>: もんだい4 試合に 勝ったら、 みんなで (   ).</t>
+          <t>: もんだい4もし お金が 足りなかったら、 アルバイトを (   ).</t>
         </is>
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t>1. お祝いすることにした 2. お祝いしたがる 3. お祝いしようと思う 4. お祝いするそうだ</t>
+          <t>1. することにした 2. したいかもしれない 3. するようになった 4. したらしい</t>
         </is>
       </c>
       <c r="D40" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E40" s="1" t="inlineStr"/>
@@ -1406,12 +1403,12 @@
       </c>
       <c r="B41" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 雨が降る (   )、試合は中止になります。</t>
+          <t>: もんだい4試合に 勝ったら、 みんなで (   ).</t>
         </is>
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
-          <t>1. から 2. なら 3. と 4. ほど</t>
+          <t>1. お祝いすることにした 2. お祝いしたがる 3. お祝いしようと思う 4. お祝いするそうだ</t>
         </is>
       </c>
       <c r="D41" s="1" t="inlineStr">
@@ -1430,17 +1427,17 @@
       </c>
       <c r="B42" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 彼が来る (   )、パーティーを始めます。</t>
+          <t>: もんだい5雨が降る (   )、試合は中止になります。</t>
         </is>
       </c>
       <c r="C42" s="1" t="inlineStr">
         <is>
-          <t>1. ので 2. と 3. ほど 4. なら</t>
+          <t>1. から 2. なら 3. と 4. ほど</t>
         </is>
       </c>
       <c r="D42" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E42" s="1" t="inlineStr"/>
@@ -1454,17 +1451,17 @@
       </c>
       <c r="B43" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 お金を持っている (   )、買い物に行けます。</t>
+          <t>: もんだい5彼が来る (   )、パーティーを始めます。</t>
         </is>
       </c>
       <c r="C43" s="1" t="inlineStr">
         <is>
-          <t>1. なら 2. ほど 3. と 4. から</t>
+          <t>1. ので 2. と 3. ほど 4. なら</t>
         </is>
       </c>
       <c r="D43" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E43" s="1" t="inlineStr"/>
@@ -1478,17 +1475,17 @@
       </c>
       <c r="B44" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 時間がある (   )、映画を見に行きましょう。</t>
+          <t>: もんだい5お金を持っている (   )、買い物に行けます。</t>
         </is>
       </c>
       <c r="C44" s="1" t="inlineStr">
         <is>
-          <t>1. と 2. から 3. ほど 4. なら</t>
+          <t>1. なら 2. ほど 3. と 4. から</t>
         </is>
       </c>
       <c r="D44" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E44" s="1" t="inlineStr"/>
@@ -1502,17 +1499,17 @@
       </c>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 このボタンを押す (   )、ドアが開きます。</t>
+          <t>: もんだい5時間がある (   )、映画を見に行きましょう。</t>
         </is>
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t>1. から 2. と 3. ほど 4. なら</t>
+          <t>1. と 2. から 3. ほど 4. なら</t>
         </is>
       </c>
       <c r="D45" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E45" s="1" t="inlineStr"/>
@@ -1526,17 +1523,17 @@
       </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 朝ごはんを食べる (   )、元気が出ます。</t>
+          <t>: もんだい5このボタンを押す (   )、ドアが開きます。</t>
         </is>
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t>1. ほど 2. なら 3. と 4. から</t>
+          <t>1. から 2. と 3. ほど 4. なら</t>
         </is>
       </c>
       <c r="D46" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E46" s="1" t="inlineStr"/>
@@ -1550,17 +1547,17 @@
       </c>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 電話をかける (   )、彼はすぐ来ます。</t>
+          <t>: もんだい5朝ごはんを食べる (   )、元気が出ます。</t>
         </is>
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t>1. ほど 2. と 3. から 4. なら</t>
+          <t>1. ほど 2. なら 3. と 4. から</t>
         </is>
       </c>
       <c r="D47" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E47" s="1" t="inlineStr"/>
@@ -1574,17 +1571,17 @@
       </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 春になる (   )、桜が咲きます。</t>
+          <t>: もんだい5電話をかける (   )、彼はすぐ来ます。</t>
         </is>
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
-          <t>1. と 2. から 3. ほど 4. なら</t>
+          <t>1. ほど 2. と 3. から 4. なら</t>
         </is>
       </c>
       <c r="D48" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E48" s="1" t="inlineStr"/>
@@ -1598,17 +1595,17 @@
       </c>
       <c r="B49" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 この薬を飲む (   )、風邪が治ります。</t>
+          <t>: もんだい5春になる (   )、桜が咲きます。</t>
         </is>
       </c>
       <c r="C49" s="1" t="inlineStr">
         <is>
-          <t>1. から 2. と 3. ほど 4. なら</t>
+          <t>1. と 2. から 3. ほど 4. なら</t>
         </is>
       </c>
       <c r="D49" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E49" s="1" t="inlineStr"/>
@@ -1622,17 +1619,17 @@
       </c>
       <c r="B50" s="1" t="inlineStr">
         <is>
-          <t>: もんだい5 音楽を聞く (   )、気分が良くなります。</t>
+          <t>: もんだい5この薬を飲む (   )、風邪が治ります。</t>
         </is>
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t>1. から 2. ほど 3. と 4. なら</t>
+          <t>1. から 2. と 3. ほど 4. なら</t>
         </is>
       </c>
       <c r="D50" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E50" s="1" t="inlineStr"/>
@@ -1646,17 +1643,17 @@
       </c>
       <c r="B51" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「このボタンをおすと どうなりますか。 」 B:「ドアが (   )。 」</t>
+          <t>: もんだい5音楽を聞く (   )、気分が良くなります。</t>
         </is>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
-          <t>1. ひらきます 2. しまります 3. とまりません 4. うごきません</t>
+          <t>1. から 2. ほど 3. と 4. なら</t>
         </is>
       </c>
       <c r="D51" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E51" s="1" t="inlineStr"/>
@@ -1670,17 +1667,17 @@
       </c>
       <c r="B52" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「雨がふると かさを(   )。 」 B:「そうですね。 」</t>
+          <t>: もんだい6A:「このボタンをおすと どうなりますか。 」 B:「ドアが (   )。 」</t>
         </is>
       </c>
       <c r="C52" s="1" t="inlineStr">
         <is>
-          <t>1. つかわなくなります 2. つかうようになります 3. つかってはいけません 4. つかいたくなくなります</t>
+          <t>1. ひらきます 2. しまります 3. とまりません 4. うごきません</t>
         </is>
       </c>
       <c r="D52" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E52" s="1" t="inlineStr"/>
@@ -1694,17 +1691,17 @@
       </c>
       <c r="B53" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「この薬を飲むと、どうなりますか。 」 B:「すぐに (   )。 」</t>
+          <t>: もんだい6A:「雨がふると かさを(   )。 」 B:「そうですね。 」</t>
         </is>
       </c>
       <c r="C53" s="1" t="inlineStr">
         <is>
-          <t>1. なおります 2. ねむくなります 3. いたくなります 4. わるくなります</t>
+          <t>1. つかわなくなります 2. つかうようになります 3. つかってはいけません 4. つかいたくなくなります</t>
         </is>
       </c>
       <c r="D53" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E53" s="1" t="inlineStr"/>
@@ -1718,12 +1715,12 @@
       </c>
       <c r="B54" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「お金を入れると ジュースが(   )。 」 B:「わかりました。 」</t>
+          <t>: もんだい6A:「この薬を飲むと、どうなりますか。 」 B:「すぐに (   )。 」</t>
         </is>
       </c>
       <c r="C54" s="1" t="inlineStr">
         <is>
-          <t>1. 出てきます 2. 出ません 3. 出にくくなります 4. 出すぎます</t>
+          <t>1. なおります 2. ねむくなります 3. いたくなります 4. わるくなります</t>
         </is>
       </c>
       <c r="D54" s="1" t="inlineStr">
@@ -1742,12 +1739,12 @@
       </c>
       <c r="B55" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「この道をまっすぐ行くと、右に何がありますか。 」 B:「(   )。 」</t>
+          <t>: もんだい6A:「お金を入れると ジュースが(   )。 」 B:「わかりました。 」</t>
         </is>
       </c>
       <c r="C55" s="1" t="inlineStr">
         <is>
-          <t>1. コンビニがあります 2. コンビニがありません 3. コンビニが見えません 4. コンビニが消えます</t>
+          <t>1. 出てきます 2. 出ません 3. 出にくくなります 4. 出すぎます</t>
         </is>
       </c>
       <c r="D55" s="1" t="inlineStr">
@@ -1766,12 +1763,12 @@
       </c>
       <c r="B56" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「天気がいいと、何をしますか。 」 B:「公園で(   )。 」</t>
+          <t>: もんだい6A:「この道をまっすぐ行くと、右に何がありますか。 」 B:「(   )。 」</t>
         </is>
       </c>
       <c r="C56" s="1" t="inlineStr">
         <is>
-          <t>1. あそびます 2. あそびません 3. あそびたくなくなります 4. あそびにくくなります</t>
+          <t>1. コンビニがあります 2. コンビニがありません 3. コンビニが見えません 4. コンビニが消えます</t>
         </is>
       </c>
       <c r="D56" s="1" t="inlineStr">
@@ -1790,12 +1787,12 @@
       </c>
       <c r="B57" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「日本に行くと、日本語が(   )。 」 B:「そうですね。 」</t>
+          <t>: もんだい6A:「天気がいいと、何をしますか。 」 B:「公園で(   )。 」</t>
         </is>
       </c>
       <c r="C57" s="1" t="inlineStr">
         <is>
-          <t>1. 上手になります 2. 下手になります 3. わからなくなります 4. 使えなくなります</t>
+          <t>1. あそびます 2. あそびません 3. あそびたくなくなります 4. あそびにくくなります</t>
         </is>
       </c>
       <c r="D57" s="1" t="inlineStr">
@@ -1814,12 +1811,12 @@
       </c>
       <c r="B58" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「このボタンをおすと、どうなるの？ 」 B:「テレビが(   )。 」</t>
+          <t>: もんだい6A:「日本に行くと、日本語が(   )。 」 B:「そうですね。 」</t>
         </is>
       </c>
       <c r="C58" s="1" t="inlineStr">
         <is>
-          <t>1. つきます 2. つかなくなります 3. けせません 4. とまりません</t>
+          <t>1. 上手になります 2. 下手になります 3. わからなくなります 4. 使えなくなります</t>
         </is>
       </c>
       <c r="D58" s="1" t="inlineStr">
@@ -1838,12 +1835,12 @@
       </c>
       <c r="B59" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「夜になると、どうなる？ 」 B:「道が(   )。 」</t>
+          <t>: もんだい6A:「このボタンをおすと、どうなるの？ 」 B:「テレビが(   )。 」</t>
         </is>
       </c>
       <c r="C59" s="1" t="inlineStr">
         <is>
-          <t>1. くらくなります 2. 明るくなります 3. さむくなります 4. あたたかくなります</t>
+          <t>1. つきます 2. つかなくなります 3. けせません 4. とまりません</t>
         </is>
       </c>
       <c r="D59" s="1" t="inlineStr">
@@ -1862,12 +1859,12 @@
       </c>
       <c r="B60" s="1" t="inlineStr">
         <is>
-          <t>: もんだい6 A:「お金がたくさんあると、どうしますか。 」 B:「旅行に(   )。 」</t>
+          <t>: もんだい6A:「夜になると、どうなる？ 」 B:「道が(   )。 」</t>
         </is>
       </c>
       <c r="C60" s="1" t="inlineStr">
         <is>
-          <t>1. 行きます 2. 行きません 3. 行きたくなくなります 4. 行けません</t>
+          <t>1. くらくなります 2. 明るくなります 3. さむくなります 4. あたたかくなります</t>
         </is>
       </c>
       <c r="D60" s="1" t="inlineStr">
@@ -1886,17 +1883,17 @@
       </c>
       <c r="B61" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 雨が降ると、(   )。</t>
+          <t>: もんだい6A:「お金がたくさんあると、どうしますか。 」 B:「旅行に(   )。 」</t>
         </is>
       </c>
       <c r="C61" s="1" t="inlineStr">
         <is>
-          <t>1. かさを持って行く 2. 外で遊べる 3. ぬれる 4. かさがない</t>
+          <t>1. 行きます 2. 行きません 3. 行きたくなくなります 4. 行けません</t>
         </is>
       </c>
       <c r="D61" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E61" s="1" t="inlineStr"/>
@@ -1910,17 +1907,17 @@
       </c>
       <c r="B62" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 毎日運動をすると、(   )。</t>
+          <t>: もんだい7雨が降ると、(   )。</t>
         </is>
       </c>
       <c r="C62" s="1" t="inlineStr">
         <is>
-          <t>1. 健康になる 2. 病気になる 3. 疲れない 4. 眠くなる</t>
+          <t>1. かさを持って行く 2. 外で遊べる 3. ぬれる 4. かさがない</t>
         </is>
       </c>
       <c r="D62" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E62" s="1" t="inlineStr"/>
@@ -1934,12 +1931,12 @@
       </c>
       <c r="B63" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 このボタンを押すと、(   )。</t>
+          <t>: もんだい7毎日運動をすると、(   )。</t>
         </is>
       </c>
       <c r="C63" s="1" t="inlineStr">
         <is>
-          <t>1. 電気がつく 2. 電気が消える 3. 音が聞こえない 4. 音が聞こえる</t>
+          <t>1. 健康になる 2. 病気になる 3. 疲れない 4. 眠くなる</t>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
@@ -1958,17 +1955,17 @@
       </c>
       <c r="B64" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 夏になると、(   )。</t>
+          <t>: もんだい7このボタンを押すと、(   )。</t>
         </is>
       </c>
       <c r="C64" s="1" t="inlineStr">
         <is>
-          <t>1. 雪が降る 2. 海に行きたくなる 3. 寒くなる 4. 外でスキーをする</t>
+          <t>1. 電気がつく 2. 電気が消える 3. 音が聞こえない 4. 音が聞こえる</t>
         </is>
       </c>
       <c r="D64" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E64" s="1" t="inlineStr"/>
@@ -1982,17 +1979,17 @@
       </c>
       <c r="B65" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 勉強しないと、(   )。</t>
+          <t>: もんだい7夏になると、(   )。</t>
         </is>
       </c>
       <c r="C65" s="1" t="inlineStr">
         <is>
-          <t>1. テストに合格する 2. テストでいい点を取る 3. テストで失敗する 4. テストを受けない</t>
+          <t>1. 雪が降る 2. 海に行きたくなる 3. 寒くなる 4. 外でスキーをする</t>
         </is>
       </c>
       <c r="D65" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E65" s="1" t="inlineStr"/>
@@ -2006,12 +2003,12 @@
       </c>
       <c r="B66" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 冬になると、(   )。</t>
+          <t>: もんだい7勉強しないと、(   )。</t>
         </is>
       </c>
       <c r="C66" s="1" t="inlineStr">
         <is>
-          <t>1. 暑くなる 2. 暖かくなる 3. 寒くなる 4. 海で泳ぐ</t>
+          <t>1. テストに合格する 2. テストでいい点を取る 3. テストで失敗する 4. テストを受けない</t>
         </is>
       </c>
       <c r="D66" s="1" t="inlineStr">
@@ -2030,17 +2027,17 @@
       </c>
       <c r="B67" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 時間があるときは、(   )。</t>
+          <t>: もんだい7冬になると、(   )。</t>
         </is>
       </c>
       <c r="C67" s="1" t="inlineStr">
         <is>
-          <t>1. 映画を見に行く 2. 忙しくなる 3. 仕事をする 4. 電車に乗らない</t>
+          <t>1. 暑くなる 2. 暖かくなる 3. 寒くなる 4. 海で泳ぐ</t>
         </is>
       </c>
       <c r="D67" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E67" s="1" t="inlineStr"/>
@@ -2054,17 +2051,17 @@
       </c>
       <c r="B68" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 お金がないと、(   )。</t>
+          <t>: もんだい7時間があるときは、(   )。</t>
         </is>
       </c>
       <c r="C68" s="1" t="inlineStr">
         <is>
-          <t>1. 買い物ができる 2. 買い物ができない 3. 旅行に行ける 4. 贅沢ができる</t>
+          <t>1. 映画を見に行く 2. 忙しくなる 3. 仕事をする 4. 電車に乗らない</t>
         </is>
       </c>
       <c r="D68" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E68" s="1" t="inlineStr"/>
@@ -2078,17 +2075,17 @@
       </c>
       <c r="B69" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 毎日日本語を勉強すると、(   )。</t>
+          <t>: もんだい7お金がないと、(   )。</t>
         </is>
       </c>
       <c r="C69" s="1" t="inlineStr">
         <is>
-          <t>1. 上手になる 2. 忘れる 3. 難しくなる 4. 話せない</t>
+          <t>1. 買い物ができる 2. 買い物ができない 3. 旅行に行ける 4. 贅沢ができる</t>
         </is>
       </c>
       <c r="D69" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E69" s="1" t="inlineStr"/>
@@ -2102,17 +2099,17 @@
       </c>
       <c r="B70" s="1" t="inlineStr">
         <is>
-          <t>: もんだい7 練習を続けると、(   )。</t>
+          <t>: もんだい7毎日日本語を勉強すると、(   )。</t>
         </is>
       </c>
       <c r="C70" s="1" t="inlineStr">
         <is>
-          <t>1. 上達しない 2. 上達する 3. もっと難しくなる 4. 興味がなくなる</t>
+          <t>1. 上手になる 2. 忘れる 3. 難しくなる 4. 話せない</t>
         </is>
       </c>
       <c r="D70" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E70" s="1" t="inlineStr"/>
@@ -2126,17 +2123,17 @@
       </c>
       <c r="B71" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 雨が降る (ふる) と (   )、気温 (きおん) が下がる。</t>
+          <t>: もんだい7練習を続けると、(   )。</t>
         </is>
       </c>
       <c r="C71" s="1" t="inlineStr">
         <is>
-          <t>1. みたい 2. らしく 3. ように 4. ほどに</t>
+          <t>1. 上達しない 2. 上達する 3. もっと難しくなる 4. 興味がなくなる</t>
         </is>
       </c>
       <c r="D71" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E71" s="1" t="inlineStr"/>
@@ -2150,17 +2147,17 @@
       </c>
       <c r="B72" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 春になる (   )、花が咲きます。</t>
+          <t>: もんだい8雨が降る (ふる) と (   )、気温 (きおん) が下がる。</t>
         </is>
       </c>
       <c r="C72" s="1" t="inlineStr">
         <is>
-          <t>1. みたい 2. ように 3. ほどに 4. と</t>
+          <t>1. みたい 2. らしく 3. ように 4. ほどに</t>
         </is>
       </c>
       <c r="D72" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E72" s="1" t="inlineStr"/>
@@ -2174,17 +2171,17 @@
       </c>
       <c r="B73" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 このボタンを押す (   )、ドアが開きます。</t>
+          <t>: もんだい8春になる (   )、花が咲きます。</t>
         </is>
       </c>
       <c r="C73" s="1" t="inlineStr">
         <is>
-          <t>1. らしく 2. ように 3. と 4. みたい</t>
+          <t>1. みたい 2. ように 3. ほどに 4. と</t>
         </is>
       </c>
       <c r="D73" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E73" s="1" t="inlineStr"/>
@@ -2198,17 +2195,17 @@
       </c>
       <c r="B74" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 夜になる (   )、星が見えます。</t>
+          <t>: もんだい8このボタンを押す (   )、ドアが開きます。</t>
         </is>
       </c>
       <c r="C74" s="1" t="inlineStr">
         <is>
-          <t>1. ほどに 2. と 3. みたい 4. ように</t>
+          <t>1. らしく 2. ように 3. と 4. みたい</t>
         </is>
       </c>
       <c r="D74" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E74" s="1" t="inlineStr"/>
@@ -2222,17 +2219,17 @@
       </c>
       <c r="B75" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 朝ご飯を食べる (   )、元気になります。</t>
+          <t>: もんだい8夜になる (   )、星が見えます。</t>
         </is>
       </c>
       <c r="C75" s="1" t="inlineStr">
         <is>
-          <t>1. ように 2. みたい 3. ほどに 4. と</t>
+          <t>1. ほどに 2. と 3. みたい 4. ように</t>
         </is>
       </c>
       <c r="D75" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E75" s="1" t="inlineStr"/>
@@ -2246,17 +2243,17 @@
       </c>
       <c r="B76" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 音楽を聴く (   )、リラックスできます。</t>
+          <t>: もんだい8朝ご飯を食べる (   )、元気になります。</t>
         </is>
       </c>
       <c r="C76" s="1" t="inlineStr">
         <is>
-          <t>1. らしく 2. と 3. みたい 4. ように</t>
+          <t>1. ように 2. みたい 3. ほどに 4. と</t>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E76" s="1" t="inlineStr"/>
@@ -2270,12 +2267,12 @@
       </c>
       <c r="B77" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 部屋が静かだ (   )、よく集中できます。</t>
+          <t>: もんだい8音楽を聴く (   )、リラックスできます。</t>
         </is>
       </c>
       <c r="C77" s="1" t="inlineStr">
         <is>
-          <t>1. みたい 2. と 3. ように 4. ほどに</t>
+          <t>1. らしく 2. と 3. みたい 4. ように</t>
         </is>
       </c>
       <c r="D77" s="1" t="inlineStr">
@@ -2294,17 +2291,17 @@
       </c>
       <c r="B78" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 この薬を飲む (   )、すぐに治ります。</t>
+          <t>: もんだい8部屋が静かだ (   )、よく集中できます。</t>
         </is>
       </c>
       <c r="C78" s="1" t="inlineStr">
         <is>
-          <t>1. と 2. みたい 3. ように 4. ほどに</t>
+          <t>1. みたい 2. と 3. ように 4. ほどに</t>
         </is>
       </c>
       <c r="D78" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E78" s="1" t="inlineStr"/>
@@ -2318,17 +2315,17 @@
       </c>
       <c r="B79" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 信号が青になる (   )、渡ってください。</t>
+          <t>: もんだい8この薬を飲む (   )、すぐに治ります。</t>
         </is>
       </c>
       <c r="C79" s="1" t="inlineStr">
         <is>
-          <t>1. ように 2. みたい 3. と 4. ほどに</t>
+          <t>1. と 2. みたい 3. ように 4. ほどに</t>
         </is>
       </c>
       <c r="D79" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E79" s="1" t="inlineStr"/>
@@ -2342,25 +2339,49 @@
       </c>
       <c r="B80" s="1" t="inlineStr">
         <is>
-          <t>: もんだい8 時間がある (   )、一緒に行きませんか。</t>
+          <t>: もんだい8信号が青になる (   )、渡ってください。</t>
         </is>
       </c>
       <c r="C80" s="1" t="inlineStr">
         <is>
-          <t>1. と 2. ように 3. ほどに 4. みたい</t>
+          <t>1. ように 2. みたい 3. と 4. ほどに</t>
         </is>
       </c>
       <c r="D80" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E80" s="1" t="inlineStr"/>
       <c r="F80" s="1" t="inlineStr"/>
     </row>
+    <row r="81">
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>Q10</t>
+        </is>
+      </c>
+      <c r="B81" s="1" t="inlineStr">
+        <is>
+          <t>: もんだい8時間がある (   )、一緒に行きませんか。</t>
+        </is>
+      </c>
+      <c r="C81" s="1" t="inlineStr">
+        <is>
+          <t>1. と 2. ように 3. ほどに 4. みたい</t>
+        </is>
+      </c>
+      <c r="D81" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E81" s="1" t="inlineStr"/>
+      <c r="F81" s="1" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High_Q,Low_Q,Drop,Minor changes"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>